<commit_message>
Removed all arduino files to avoid problems and upgraded all files after Major task
</commit_message>
<xml_diff>
--- a/Project/Documentation/Parts.xlsx
+++ b/Project/Documentation/Parts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danda\BOM-project\Project\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4FE329C9-A144-4C85-B1A9-76874F430DD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{192AC1FA-B9B6-4475-8530-E66E24C00474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5DE35E3E-6C09-4D2A-8945-45C6D5772E32}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <si>
     <t xml:space="preserve">Breadboards </t>
   </si>
@@ -132,13 +132,49 @@
   </si>
   <si>
     <t xml:space="preserve">Electrical / Arduino </t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIFTING MECHANISM </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> # Needed</t>
+  </si>
+  <si>
+    <t>DC Motor</t>
+  </si>
+  <si>
+    <t>H-bridge  ( Motor Driver )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IR Sensor </t>
+  </si>
+  <si>
+    <t>Sorting Mechanism</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parts </t>
+  </si>
+  <si>
+    <t>IR sensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Micro servo Motor </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arduino Uno </t>
+  </si>
+  <si>
+    <t xml:space="preserve">H-Bridge </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -176,8 +212,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="28"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -199,6 +243,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -239,15 +289,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -258,34 +305,42 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF009900"/>
         </patternFill>
       </fill>
     </dxf>
@@ -299,21 +354,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF009900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF009900"/>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -653,139 +694,246 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59611B78-6837-4C49-98D3-EFB4E8B8C170}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr defaultColWidth="15.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" style="8"/>
+    <col min="1" max="1" width="15.33203125" style="7"/>
     <col min="3" max="3" width="15.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="A2" s="3" t="s">
+      <c r="G1" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="K1" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+    </row>
+    <row r="2" spans="1:13" ht="25.8" x14ac:dyDescent="0.5">
+      <c r="A2" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="C3" s="8">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <f>SUM(I7,M4)</f>
+        <v>3</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="14"/>
+      <c r="I3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="L3" s="14"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
         <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="C4" s="8">
+        <v>1</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" s="14"/>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="K4" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4" s="14"/>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="25.8" x14ac:dyDescent="0.5">
+      <c r="C5" s="8">
+        <v>1</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="14"/>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="K5" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="L5" s="14"/>
+      <c r="M5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="25.8" x14ac:dyDescent="0.5">
       <c r="A6" s="10" t="s">
         <v>25</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="G6" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" s="14"/>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="K6" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="L6" s="14"/>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="C7" s="8">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <f>M5</f>
+        <v>2</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7" s="14"/>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="L7" s="14"/>
+      <c r="M7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="C8" s="8">
+        <v>1</v>
+      </c>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
+      <c r="C9" s="8">
+        <v>1</v>
+      </c>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10" s="6"/>
       <c r="B10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="8">
         <v>2</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+      <c r="D10">
+        <f>I4</f>
+        <v>1</v>
+      </c>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
+      <c r="C11" s="8">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <f>I5+M7</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" s="6"/>
       <c r="B12" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:13" ht="25.8" x14ac:dyDescent="0.5">
       <c r="A13" s="12" t="s">
         <v>31</v>
       </c>
@@ -793,92 +941,110 @@
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="8">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
+      <c r="D14">
+        <f>I6+M6</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A15" s="6"/>
       <c r="B15" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="7"/>
+      <c r="A18" s="6"/>
       <c r="B18" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C18" s="9">
+      <c r="C18" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="7"/>
+      <c r="A19" s="6"/>
       <c r="B19" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="7"/>
+      <c r="A20" s="6"/>
       <c r="B20" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="8">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="19">
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="K1:M2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="K6:L6"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A13:D13"/>
+    <mergeCell ref="G1:I2"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G10:H10"/>
   </mergeCells>
   <conditionalFormatting sqref="D3:D5 D7:D12 D14:D20">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="greaterThan">
-      <formula>$C$3</formula>
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>D3&lt;C3</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D5 D7:D12 D14:D20">
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>D3&gt;=C3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="1">
-      <formula>D3&lt;C3</formula>
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="greaterThan">
+      <formula>$C$3</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>